<commit_message>
R9: read an exclusive option chosen with another as a condition
</commit_message>
<xml_diff>
--- a/out/C03_b2b_saas_decision_journey/agent3/agent3_test_cases_for_review.xlsx
+++ b/out/C03_b2b_saas_decision_journey/agent3/agent3_test_cases_for_review.xlsx
@@ -2044,7 +2044,7 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>TC-b7c7601f55</t>
+          <t>TC-f7f230fdae</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
@@ -2058,7 +2058,7 @@
 2. S2 = A decision-maker or major influencer for business software
 3. S3 = No
 4. S4 = No
-5. Q1 = None of these</t>
+5. Q1 = Open-source alternative</t>
         </is>
       </c>
       <c r="H25" s="3" t="inlineStr">
@@ -2429,7 +2429,7 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>TC-96c01d824f</t>
+          <t>TC-b41beb2f71</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
@@ -2443,7 +2443,7 @@
 2. S2 = A decision-maker or major influencer for business software
 3. S3 = No
 4. S4 = No
-5. Q1 = None of these</t>
+5. Q1 = Open-source alternative</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr">

</xml_diff>